<commit_message>
product migration module update
</commit_message>
<xml_diff>
--- a/apps/admin/public/assets/migration_sample/products-sample.xlsx
+++ b/apps/admin/public/assets/migration_sample/products-sample.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\asian-spices\apps\admin\public\assets\migration_sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{92126BF1-1530-44BC-BF8A-39F09E159E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{939FE4E9-28A4-46A2-9103-02C0FC286975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D4E227D-3D23-4167-ADF5-602103F06CAD}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="59">
   <si>
     <t>Name</t>
   </si>
@@ -193,6 +193,27 @@
   </si>
   <si>
     <t>Smartwatch with GPS</t>
+  </si>
+  <si>
+    <t>Available Countries</t>
+  </si>
+  <si>
+    <t>Health Benefits</t>
+  </si>
+  <si>
+    <t>Images</t>
+  </si>
+  <si>
+    <t>B2B Prices</t>
+  </si>
+  <si>
+    <t>Catalog Store</t>
+  </si>
+  <si>
+    <t>Catalog Price</t>
+  </si>
+  <si>
+    <t>Catalog Quantity</t>
   </si>
 </sst>
 </file>
@@ -558,19 +579,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DE05638-4344-4D50-A8BE-CC6B0971A9A1}">
-  <dimension ref="A1:N5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:U5"/>
+  <sheetFormatPr defaultColWidth="11.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.5546875" customWidth="1"/>
+    <col min="12" max="12" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.88671875" customWidth="1"/>
+    <col min="14" max="14" width="10.33203125" customWidth="1"/>
+    <col min="15" max="15" width="11.5546875" customWidth="1"/>
+    <col min="16" max="16" width="6.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -596,25 +626,46 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="Q1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
@@ -639,26 +690,28 @@
       <c r="H2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="2"/>
+      <c r="J2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="2">
+      <c r="K2" s="2"/>
+      <c r="L2" s="2">
         <v>599.99</v>
       </c>
-      <c r="K2" s="2">
+      <c r="M2" s="2">
         <v>50</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="M2" s="2">
+      <c r="O2" s="2">
         <v>10</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>25</v>
       </c>
@@ -683,26 +736,28 @@
       <c r="H3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="2"/>
+      <c r="J3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="2">
+      <c r="K3" s="2"/>
+      <c r="L3" s="2">
         <v>299.99</v>
       </c>
-      <c r="K3" s="2">
+      <c r="M3" s="2">
         <v>200</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="M3" s="2">
+      <c r="O3" s="2">
         <v>25</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="P3" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -727,26 +782,28 @@
       <c r="H4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="2"/>
+      <c r="J4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="J4" s="2">
+      <c r="K4" s="2"/>
+      <c r="L4" s="2">
         <v>120</v>
       </c>
-      <c r="K4" s="2">
+      <c r="M4" s="2">
         <v>150</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M4" s="2">
+      <c r="O4" s="2">
         <v>0</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>45</v>
       </c>
@@ -771,22 +828,24 @@
       <c r="H5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="2"/>
+      <c r="J5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="2">
+      <c r="K5" s="2"/>
+      <c r="L5" s="2">
         <v>399.99</v>
       </c>
-      <c r="K5" s="2">
+      <c r="M5" s="2">
         <v>100</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="M5" s="2">
+      <c r="O5" s="2">
         <v>5</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="P5" s="2" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>